<commit_message>
C&G: comment out redundant btn_Finish s98 (admission already finished at s96)
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/C&G/LSTP_C&G_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/C&G/LSTP_C&G_WF001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrishnan6\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\C&amp;G\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03E3597C-3BE4-42AB-A95A-87B9697E2DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCE74A7-F13C-401A-9375-E4F424CA7484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1EFC42B6-5B45-43D8-9445-5004CB3116B1}"/>
+    <workbookView xWindow="1125" yWindow="-15045" windowWidth="21600" windowHeight="11295" xr2:uid="{1EFC42B6-5B45-43D8-9445-5004CB3116B1}"/>
   </bookViews>
   <sheets>
     <sheet name="TestExecution" sheetId="1" r:id="rId1"/>
@@ -369,9 +369,6 @@
     <t>btn_Close</t>
   </si>
   <si>
-    <t>Click Finish in coding screen to complete admission workflow</t>
-  </si>
-  <si>
     <t>btn_Finish</t>
   </si>
   <si>
@@ -1165,6 +1162,9 @@
   </si>
   <si>
     <t>Wait for Coding workload</t>
+  </si>
+  <si>
+    <t>// Click Finish in coding screen to complete admission workflow</t>
   </si>
 </sst>
 </file>
@@ -1885,7 +1885,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C2" s="11" t="s">
         <v>11</v>
@@ -1917,7 +1917,7 @@
         <v>13</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1925,7 +1925,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>11</v>
@@ -1942,7 +1942,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>18</v>
@@ -1959,7 +1959,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>18</v>
@@ -1996,7 +1996,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>25</v>
@@ -2005,7 +2005,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F8" s="11" t="s">
         <v>20</v>
@@ -2057,7 +2057,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>18</v>
@@ -2066,7 +2066,7 @@
         <v>33</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F11" s="11" t="s">
         <v>20</v>
@@ -2077,34 +2077,34 @@
         <v>11</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>34</v>
       </c>
       <c r="D12" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="F12" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="E12" s="11" t="s">
-        <v>225</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>226</v>
-      </c>
       <c r="G12" s="11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -2112,7 +2112,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>34</v>
@@ -2129,7 +2129,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>34</v>
@@ -2141,7 +2141,7 @@
       <c r="H14" s="14"/>
       <c r="I14" s="14"/>
       <c r="J14" s="14" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -2149,7 +2149,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>34</v>
@@ -2169,19 +2169,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>34</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F16" s="11" t="s">
         <v>48</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -2189,19 +2189,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>34</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F17" s="11" t="s">
         <v>13</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -2209,13 +2209,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>34</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F18" s="11" t="s">
         <v>20</v>
@@ -2226,19 +2226,19 @@
         <v>18</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>34</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>13</v>
       </c>
       <c r="J19" s="15" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -2263,7 +2263,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>41</v>
@@ -2337,7 +2337,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>52</v>
@@ -2354,7 +2354,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>52</v>
@@ -2371,7 +2371,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>52</v>
@@ -2388,16 +2388,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>52</v>
       </c>
       <c r="F28" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="J28" s="11" t="s">
         <v>242</v>
-      </c>
-      <c r="J28" s="11" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
@@ -2405,16 +2405,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>52</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
@@ -2422,23 +2422,23 @@
         <v>29</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>52</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E30" s="11"/>
       <c r="F30" s="11" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G30" s="11"/>
       <c r="H30" s="11"/>
       <c r="I30" s="11"/>
       <c r="J30" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="K30" s="11"/>
       <c r="L30" s="16"/>
@@ -2448,7 +2448,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>52</v>
@@ -2456,13 +2456,13 @@
       <c r="D31" s="17"/>
       <c r="E31" s="17"/>
       <c r="F31" s="17" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G31" s="17"/>
       <c r="H31" s="17"/>
       <c r="I31" s="17"/>
       <c r="J31" s="17" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="K31" s="11"/>
       <c r="L31" s="16"/>
@@ -2472,7 +2472,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>54</v>
@@ -2492,19 +2492,19 @@
         <v>32</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>54</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F33" s="11" t="s">
         <v>13</v>
       </c>
       <c r="K33" s="11" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2529,7 +2529,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>54</v>
@@ -2546,7 +2546,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>54</v>
@@ -2580,7 +2580,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>63</v>
@@ -2597,7 +2597,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>63</v>
@@ -2614,10 +2614,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="C40" s="11" t="s">
         <v>258</v>
-      </c>
-      <c r="C40" s="11" t="s">
-        <v>259</v>
       </c>
       <c r="D40" s="11" t="s">
         <v>96</v>
@@ -2634,10 +2634,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D41" s="11" t="s">
         <v>40</v>
@@ -2651,10 +2651,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D42" s="11" t="s">
         <v>98</v>
@@ -2785,13 +2785,13 @@
         <v>48</v>
       </c>
       <c r="B49" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="F49" s="11" t="s">
         <v>262</v>
       </c>
-      <c r="F49" s="11" t="s">
+      <c r="J49" s="11" t="s">
         <v>263</v>
-      </c>
-      <c r="J49" s="11" t="s">
-        <v>264</v>
       </c>
       <c r="K49" s="5"/>
     </row>
@@ -2800,19 +2800,19 @@
         <v>49</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C50" s="11" t="s">
         <v>69</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F50" s="11" t="s">
         <v>13</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K50" s="5"/>
     </row>
@@ -2821,19 +2821,19 @@
         <v>50</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C51" s="11" t="s">
         <v>69</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F51" s="11" t="s">
         <v>13</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K51" s="5"/>
     </row>
@@ -2842,19 +2842,19 @@
         <v>51</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C52" s="11" t="s">
         <v>69</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F52" s="11" t="s">
         <v>48</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="K52" s="5"/>
     </row>
@@ -2863,7 +2863,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C53" s="11" t="s">
         <v>69</v>
@@ -2881,10 +2881,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D54" s="11" t="s">
         <v>96</v>
@@ -2893,7 +2893,7 @@
         <v>13</v>
       </c>
       <c r="J54" s="9" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="K54" s="5"/>
     </row>
@@ -2902,10 +2902,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C55" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D55" s="11" t="s">
         <v>40</v>
@@ -2920,10 +2920,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D56" s="11" t="s">
         <v>98</v>
@@ -2938,7 +2938,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C57" s="11" t="s">
         <v>52</v>
@@ -2956,7 +2956,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C58" s="11" t="s">
         <v>52</v>
@@ -2974,13 +2974,13 @@
         <v>58</v>
       </c>
       <c r="B59" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="F59" s="11" t="s">
         <v>262</v>
       </c>
-      <c r="F59" s="11" t="s">
+      <c r="J59" s="11" t="s">
         <v>263</v>
-      </c>
-      <c r="J59" s="11" t="s">
-        <v>264</v>
       </c>
       <c r="K59" s="6"/>
     </row>
@@ -2989,19 +2989,19 @@
         <v>59</v>
       </c>
       <c r="B60" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="C60" s="11" t="s">
         <v>275</v>
       </c>
-      <c r="C60" s="11" t="s">
+      <c r="D60" s="11" t="s">
         <v>276</v>
-      </c>
-      <c r="D60" s="11" t="s">
-        <v>277</v>
       </c>
       <c r="F60" s="11" t="s">
         <v>13</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K60" s="6"/>
     </row>
@@ -3010,10 +3010,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C61" s="11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F61" s="11" t="s">
         <v>85</v>
@@ -3028,13 +3028,13 @@
         <v>61</v>
       </c>
       <c r="B62" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="C62" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="D62" s="11" t="s">
         <v>278</v>
-      </c>
-      <c r="C62" s="11" t="s">
-        <v>276</v>
-      </c>
-      <c r="D62" s="11" t="s">
-        <v>279</v>
       </c>
       <c r="F62" s="11" t="s">
         <v>20</v>
@@ -3047,7 +3047,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C63" s="11" t="s">
         <v>52</v>
@@ -3063,7 +3063,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C64" s="11" t="s">
         <v>52</v>
@@ -3082,13 +3082,13 @@
         <v>64</v>
       </c>
       <c r="B65" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C65" s="11" t="s">
         <v>18</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K65" s="6"/>
       <c r="L65" s="6"/>
@@ -3098,7 +3098,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C66" s="13" t="s">
         <v>82</v>
@@ -3117,14 +3117,14 @@
         <v>66</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C67" s="13"/>
       <c r="F67" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="J67" s="11" t="s">
         <v>283</v>
-      </c>
-      <c r="J67" s="11" t="s">
-        <v>284</v>
       </c>
       <c r="K67" s="6"/>
       <c r="L67" s="6"/>
@@ -3134,7 +3134,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C68" s="13" t="s">
         <v>82</v>
@@ -3143,13 +3143,13 @@
         <v>31</v>
       </c>
       <c r="F68" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I68" s="11" t="s">
         <v>285</v>
       </c>
-      <c r="I68" s="11" t="s">
+      <c r="J68" s="11" t="s">
         <v>286</v>
-      </c>
-      <c r="J68" s="11" t="s">
-        <v>287</v>
       </c>
       <c r="K68" s="6"/>
       <c r="L68" s="6"/>
@@ -3159,7 +3159,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C69" s="13" t="s">
         <v>82</v>
@@ -3175,13 +3175,13 @@
         <v>69</v>
       </c>
       <c r="B70" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="C70" s="11" t="s">
         <v>288</v>
       </c>
-      <c r="C70" s="11" t="s">
+      <c r="D70" s="13" t="s">
         <v>289</v>
-      </c>
-      <c r="D70" s="13" t="s">
-        <v>290</v>
       </c>
       <c r="F70" s="11" t="s">
         <v>20</v>
@@ -3194,13 +3194,13 @@
         <v>70</v>
       </c>
       <c r="B71" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="C71" s="11" t="s">
         <v>291</v>
       </c>
-      <c r="C71" s="11" t="s">
+      <c r="D71" s="11" t="s">
         <v>292</v>
-      </c>
-      <c r="D71" s="11" t="s">
-        <v>293</v>
       </c>
       <c r="F71" s="11" t="s">
         <v>20</v>
@@ -3213,10 +3213,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F72" s="11" t="s">
         <v>85</v>
@@ -3232,25 +3232,25 @@
         <v>72</v>
       </c>
       <c r="B73" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="C73" s="11" t="s">
         <v>291</v>
       </c>
-      <c r="C73" s="11" t="s">
-        <v>292</v>
-      </c>
       <c r="D73" s="11" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F73" s="11" t="s">
         <v>83</v>
       </c>
       <c r="G73" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="H73" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="J73" s="11" t="s">
         <v>295</v>
-      </c>
-      <c r="H73" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="J73" s="11" t="s">
-        <v>296</v>
       </c>
       <c r="K73" s="8"/>
       <c r="L73" s="8"/>
@@ -3260,13 +3260,13 @@
         <v>73</v>
       </c>
       <c r="B74" s="11" t="s">
+        <v>296</v>
+      </c>
+      <c r="C74" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="D74" s="11" t="s">
         <v>297</v>
-      </c>
-      <c r="C74" s="11" t="s">
-        <v>289</v>
-      </c>
-      <c r="D74" s="11" t="s">
-        <v>298</v>
       </c>
       <c r="F74" s="11" t="s">
         <v>20</v>
@@ -3279,7 +3279,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C75" s="11" t="s">
         <v>18</v>
@@ -3299,13 +3299,13 @@
         <v>75</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C76" s="11" t="s">
         <v>18</v>
       </c>
       <c r="D76" s="11" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F76" s="11" t="s">
         <v>20</v>
@@ -3316,19 +3316,19 @@
         <v>76</v>
       </c>
       <c r="B77" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="C77" s="11" t="s">
         <v>301</v>
       </c>
-      <c r="C77" s="11" t="s">
+      <c r="D77" s="11" t="s">
         <v>302</v>
-      </c>
-      <c r="D77" s="11" t="s">
-        <v>303</v>
       </c>
       <c r="F77" s="11" t="s">
         <v>48</v>
       </c>
       <c r="J77" s="11" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.25">
@@ -3336,19 +3336,19 @@
         <v>77</v>
       </c>
       <c r="B78" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="C78" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="D78" s="11" t="s">
         <v>304</v>
-      </c>
-      <c r="C78" s="11" t="s">
-        <v>302</v>
-      </c>
-      <c r="D78" s="11" t="s">
-        <v>305</v>
       </c>
       <c r="F78" s="11" t="s">
         <v>48</v>
       </c>
       <c r="J78" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
@@ -3356,10 +3356,10 @@
         <v>78</v>
       </c>
       <c r="B79" s="11" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C79" s="11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D79" s="11" t="s">
         <v>81</v>
@@ -3373,13 +3373,13 @@
         <v>79</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C80" s="11" t="s">
         <v>25</v>
       </c>
       <c r="F80" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
@@ -3387,7 +3387,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="11" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C81" s="13" t="s">
         <v>82</v>
@@ -3404,14 +3404,14 @@
         <v>81</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C82" s="13"/>
       <c r="F82" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="J82" s="11" t="s">
         <v>283</v>
-      </c>
-      <c r="J82" s="11" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
@@ -3419,7 +3419,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C83" s="13" t="s">
         <v>82</v>
@@ -3428,13 +3428,13 @@
         <v>31</v>
       </c>
       <c r="F83" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I83" s="11" t="s">
         <v>285</v>
       </c>
-      <c r="I83" s="11" t="s">
+      <c r="J83" s="11" t="s">
         <v>286</v>
-      </c>
-      <c r="J83" s="11" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
@@ -3442,13 +3442,13 @@
         <v>83</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C84" s="13" t="s">
         <v>82</v>
       </c>
       <c r="F84" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
@@ -3456,13 +3456,13 @@
         <v>84</v>
       </c>
       <c r="B85" s="11" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C85" s="11" t="s">
         <v>18</v>
       </c>
       <c r="F85" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
@@ -3470,13 +3470,13 @@
         <v>85</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C86" s="11" t="s">
         <v>18</v>
       </c>
       <c r="D86" s="11" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F86" s="11" t="s">
         <v>20</v>
@@ -3487,13 +3487,13 @@
         <v>86</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C87" s="11" t="s">
         <v>18</v>
       </c>
       <c r="F87" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
@@ -3501,19 +3501,19 @@
         <v>87</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C88" s="11" t="s">
         <v>18</v>
       </c>
       <c r="F88" s="12" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G88" s="12"/>
       <c r="H88" s="12"/>
       <c r="I88" s="12"/>
       <c r="J88" s="12" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
@@ -3521,13 +3521,13 @@
         <v>88</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C89" s="12" t="s">
         <v>94</v>
       </c>
       <c r="F89" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
@@ -3547,7 +3547,7 @@
         <v>48</v>
       </c>
       <c r="J90" s="11" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
@@ -3567,7 +3567,7 @@
         <v>48</v>
       </c>
       <c r="J91" s="11" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="92" spans="1:10" ht="19.5" x14ac:dyDescent="0.25">
@@ -3581,14 +3581,14 @@
         <v>94</v>
       </c>
       <c r="D92" s="11" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E92" s="18"/>
       <c r="F92" s="11" t="s">
         <v>48</v>
       </c>
       <c r="J92" s="11" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
@@ -3613,13 +3613,13 @@
         <v>93</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C94" s="12" t="s">
         <v>94</v>
       </c>
       <c r="F94" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
@@ -3639,7 +3639,7 @@
         <v>48</v>
       </c>
       <c r="J95" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
@@ -3659,7 +3659,7 @@
         <v>48</v>
       </c>
       <c r="J96" s="11" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
@@ -3667,7 +3667,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="11" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C97" s="11" t="s">
         <v>94</v>
@@ -3684,7 +3684,7 @@
         <v>97</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C98" s="11" t="s">
         <v>103</v>
@@ -3701,13 +3701,13 @@
         <v>98</v>
       </c>
       <c r="B99" s="11" t="s">
-        <v>105</v>
+        <v>370</v>
       </c>
       <c r="C99" s="11" t="s">
         <v>103</v>
       </c>
       <c r="D99" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F99" s="11" t="s">
         <v>20</v>
@@ -3718,13 +3718,13 @@
         <v>99</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C100" s="11" t="s">
         <v>18</v>
       </c>
       <c r="F100" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
@@ -3732,13 +3732,13 @@
         <v>100</v>
       </c>
       <c r="B101" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C101" s="11" t="s">
         <v>18</v>
       </c>
       <c r="F101" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
@@ -3746,7 +3746,7 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F102" t="s">
         <v>85</v>
@@ -3760,13 +3760,13 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C103" t="s">
         <v>18</v>
       </c>
       <c r="D103" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F103" t="s">
         <v>20</v>
@@ -3777,13 +3777,13 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
+        <v>109</v>
+      </c>
+      <c r="C104" t="s">
         <v>110</v>
       </c>
-      <c r="C104" t="s">
+      <c r="F104" t="s">
         <v>111</v>
-      </c>
-      <c r="F104" t="s">
-        <v>112</v>
       </c>
       <c r="J104">
         <v>2</v>
@@ -3794,13 +3794,13 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C105" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D105" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="F105" t="s">
         <v>48</v>
@@ -3814,13 +3814,13 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C106" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D106" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F106" t="s">
         <v>20</v>
@@ -3831,13 +3831,13 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C107" t="s">
         <v>18</v>
       </c>
       <c r="D107" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F107" t="s">
         <v>20</v>
@@ -3848,19 +3848,19 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C108" t="s">
         <v>18</v>
       </c>
       <c r="D108" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F108" t="s">
         <v>13</v>
       </c>
       <c r="J108" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.25">
@@ -3868,13 +3868,13 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C109" t="s">
         <v>18</v>
       </c>
       <c r="D109" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F109" t="s">
         <v>20</v>
@@ -3885,13 +3885,13 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C110" t="s">
+        <v>110</v>
+      </c>
+      <c r="F110" t="s">
         <v>111</v>
-      </c>
-      <c r="F110" t="s">
-        <v>112</v>
       </c>
       <c r="J110">
         <v>2</v>
@@ -3902,13 +3902,13 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C111" t="s">
         <v>18</v>
       </c>
       <c r="D111" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F111" t="s">
         <v>20</v>
@@ -3919,19 +3919,19 @@
         <v>111</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C112" s="21"/>
       <c r="D112" s="22"/>
       <c r="E112" s="6"/>
       <c r="F112" s="6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G112" s="6"/>
       <c r="H112" s="6"/>
       <c r="I112" s="6"/>
       <c r="J112" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
@@ -3939,13 +3939,13 @@
         <v>112</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C113" s="21" t="s">
         <v>18</v>
       </c>
       <c r="D113" s="23" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E113" s="6"/>
       <c r="F113" t="s">
@@ -3961,13 +3961,13 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C114" t="s">
+        <v>110</v>
+      </c>
+      <c r="F114" t="s">
         <v>111</v>
-      </c>
-      <c r="F114" t="s">
-        <v>112</v>
       </c>
       <c r="J114">
         <v>2</v>
@@ -3978,13 +3978,13 @@
         <v>114</v>
       </c>
       <c r="B115" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="C115" s="21" t="s">
         <v>359</v>
       </c>
-      <c r="C115" s="21" t="s">
+      <c r="D115" s="23" t="s">
         <v>360</v>
-      </c>
-      <c r="D115" s="23" t="s">
-        <v>361</v>
       </c>
       <c r="E115" s="6"/>
       <c r="F115" t="s">
@@ -4000,13 +4000,13 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C116" t="s">
+        <v>110</v>
+      </c>
+      <c r="F116" t="s">
         <v>111</v>
-      </c>
-      <c r="F116" t="s">
-        <v>112</v>
       </c>
       <c r="J116">
         <v>2</v>
@@ -4017,13 +4017,13 @@
         <v>116</v>
       </c>
       <c r="B117" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="C117" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="D117" s="23" t="s">
         <v>336</v>
-      </c>
-      <c r="C117" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="D117" s="23" t="s">
-        <v>337</v>
       </c>
       <c r="E117" s="6"/>
       <c r="F117" t="s">
@@ -4039,13 +4039,13 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
+        <v>114</v>
+      </c>
+      <c r="C118" t="s">
+        <v>110</v>
+      </c>
+      <c r="D118" t="s">
         <v>115</v>
-      </c>
-      <c r="C118" t="s">
-        <v>111</v>
-      </c>
-      <c r="D118" t="s">
-        <v>116</v>
       </c>
       <c r="F118" t="s">
         <v>20</v>
@@ -4056,13 +4056,13 @@
         <v>118</v>
       </c>
       <c r="B119" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C119" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="D119" s="23" t="s">
         <v>338</v>
-      </c>
-      <c r="C119" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="D119" s="23" t="s">
-        <v>339</v>
       </c>
       <c r="F119" s="6" t="s">
         <v>20</v>
@@ -4073,13 +4073,13 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
+        <v>116</v>
+      </c>
+      <c r="C120" t="s">
         <v>117</v>
       </c>
-      <c r="C120" t="s">
-        <v>118</v>
-      </c>
       <c r="F120" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.25">
@@ -4087,7 +4087,7 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F121" t="s">
         <v>85</v>
@@ -4101,13 +4101,13 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C122" t="s">
         <v>18</v>
       </c>
       <c r="D122" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F122" t="s">
         <v>20</v>
@@ -4118,13 +4118,13 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C123" t="s">
         <v>18</v>
       </c>
       <c r="D123" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F123" t="s">
         <v>20</v>
@@ -4135,13 +4135,13 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C124" t="s">
         <v>18</v>
       </c>
       <c r="F124" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J124">
         <v>2</v>
@@ -4152,13 +4152,13 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C125" t="s">
         <v>18</v>
       </c>
       <c r="D125" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F125" t="s">
         <v>20</v>
@@ -4169,7 +4169,7 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C126" t="s">
         <v>18</v>
@@ -4186,13 +4186,13 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C127" t="s">
         <v>18</v>
       </c>
       <c r="D127" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="F127" t="s">
         <v>20</v>
@@ -4203,7 +4203,7 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F128" t="s">
         <v>85</v>
@@ -4217,19 +4217,19 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C129" t="s">
         <v>18</v>
       </c>
       <c r="D129" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F129" t="s">
         <v>20</v>
       </c>
       <c r="J129" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.25">
@@ -4237,7 +4237,7 @@
         <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F130" t="s">
         <v>85</v>
@@ -4251,13 +4251,13 @@
         <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C131" t="s">
         <v>18</v>
       </c>
       <c r="D131" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F131" t="s">
         <v>20</v>
@@ -4268,19 +4268,19 @@
         <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C132" t="s">
         <v>18</v>
       </c>
       <c r="D132" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F132" t="s">
         <v>13</v>
       </c>
       <c r="J132" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.25">
@@ -4288,13 +4288,13 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C133" t="s">
         <v>18</v>
       </c>
       <c r="D133" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F133" t="s">
         <v>20</v>
@@ -4305,19 +4305,19 @@
         <v>133</v>
       </c>
       <c r="B134" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C134" t="s">
         <v>18</v>
       </c>
       <c r="D134" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F134" t="s">
         <v>48</v>
       </c>
       <c r="J134" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.25">
@@ -4325,13 +4325,13 @@
         <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C135" t="s">
         <v>18</v>
       </c>
       <c r="D135" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F135" t="s">
         <v>20</v>
@@ -4342,13 +4342,13 @@
         <v>135</v>
       </c>
       <c r="B136" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C136" t="s">
         <v>18</v>
       </c>
       <c r="F136" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.25">
@@ -4356,13 +4356,13 @@
         <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C137" t="s">
         <v>18</v>
       </c>
       <c r="D137" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F137" t="s">
         <v>83</v>
@@ -4371,7 +4371,7 @@
         <v>84</v>
       </c>
       <c r="H137" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J137" t="b">
         <v>1</v>
@@ -4382,7 +4382,7 @@
         <v>137</v>
       </c>
       <c r="B138" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F138" t="s">
         <v>85</v>
@@ -4396,13 +4396,13 @@
         <v>138</v>
       </c>
       <c r="B139" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C139" t="s">
         <v>18</v>
       </c>
       <c r="D139" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F139" t="s">
         <v>20</v>
@@ -4413,13 +4413,13 @@
         <v>139</v>
       </c>
       <c r="B140" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C140" t="s">
         <v>18</v>
       </c>
       <c r="D140" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F140" t="s">
         <v>20</v>
@@ -4430,13 +4430,13 @@
         <v>140</v>
       </c>
       <c r="B141" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C141" t="s">
         <v>18</v>
       </c>
       <c r="F141" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J141">
         <v>2</v>
@@ -4447,7 +4447,7 @@
         <v>141</v>
       </c>
       <c r="B142" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C142" t="s">
         <v>18</v>
@@ -4464,13 +4464,13 @@
         <v>142</v>
       </c>
       <c r="B143" t="s">
+        <v>342</v>
+      </c>
+      <c r="C143" t="s">
+        <v>141</v>
+      </c>
+      <c r="D143" t="s">
         <v>343</v>
-      </c>
-      <c r="C143" t="s">
-        <v>142</v>
-      </c>
-      <c r="D143" t="s">
-        <v>344</v>
       </c>
       <c r="F143" t="s">
         <v>20</v>
@@ -4481,7 +4481,7 @@
         <v>143</v>
       </c>
       <c r="B144" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F144" t="s">
         <v>85</v>
@@ -4495,19 +4495,19 @@
         <v>144</v>
       </c>
       <c r="B145" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C145" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D145" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F145" t="s">
         <v>20</v>
       </c>
       <c r="J145" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.25">
@@ -4515,13 +4515,13 @@
         <v>145</v>
       </c>
       <c r="B146" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C146" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D146" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F146" t="s">
         <v>20</v>
@@ -4532,19 +4532,19 @@
         <v>146</v>
       </c>
       <c r="B147" t="s">
+        <v>347</v>
+      </c>
+      <c r="C147" t="s">
+        <v>141</v>
+      </c>
+      <c r="D147" t="s">
         <v>348</v>
-      </c>
-      <c r="C147" t="s">
-        <v>142</v>
-      </c>
-      <c r="D147" t="s">
-        <v>349</v>
       </c>
       <c r="F147" t="s">
         <v>13</v>
       </c>
       <c r="J147" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.25">
@@ -4552,13 +4552,13 @@
         <v>147</v>
       </c>
       <c r="B148" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C148" t="s">
         <v>18</v>
       </c>
       <c r="D148" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F148" t="s">
         <v>20</v>
@@ -4569,13 +4569,13 @@
         <v>148</v>
       </c>
       <c r="B149" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C149" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D149" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="F149" t="s">
         <v>20</v>
@@ -4586,13 +4586,13 @@
         <v>149</v>
       </c>
       <c r="B150" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C150" t="s">
         <v>18</v>
       </c>
       <c r="F150" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.25">
@@ -4600,13 +4600,13 @@
         <v>150</v>
       </c>
       <c r="B151" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C151" t="s">
         <v>18</v>
       </c>
       <c r="D151" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F151" t="s">
         <v>83</v>
@@ -4615,7 +4615,7 @@
         <v>84</v>
       </c>
       <c r="H151" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J151" t="b">
         <v>1</v>
@@ -4626,7 +4626,7 @@
         <v>151</v>
       </c>
       <c r="B152" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F152" t="s">
         <v>85</v>
@@ -4640,13 +4640,13 @@
         <v>152</v>
       </c>
       <c r="B153" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C153" t="s">
         <v>18</v>
       </c>
       <c r="F153" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J153">
         <v>2</v>
@@ -4657,13 +4657,13 @@
         <v>153</v>
       </c>
       <c r="B154" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C154" t="s">
         <v>18</v>
       </c>
       <c r="D154" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F154" t="s">
         <v>20</v>
@@ -4674,13 +4674,13 @@
         <v>154</v>
       </c>
       <c r="B155" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C155" t="s">
         <v>18</v>
       </c>
       <c r="D155" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F155" t="s">
         <v>20</v>
@@ -4691,13 +4691,13 @@
         <v>155</v>
       </c>
       <c r="B156" t="s">
+        <v>150</v>
+      </c>
+      <c r="C156" t="s">
         <v>151</v>
       </c>
-      <c r="C156" t="s">
-        <v>152</v>
-      </c>
       <c r="F156" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.25">
@@ -4705,10 +4705,10 @@
         <v>156</v>
       </c>
       <c r="B157" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C157" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D157" t="s">
         <v>61</v>
@@ -4722,10 +4722,10 @@
         <v>157</v>
       </c>
       <c r="B158" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C158" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D158" t="s">
         <v>104</v>
@@ -4739,13 +4739,13 @@
         <v>158</v>
       </c>
       <c r="B159" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C159" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D159" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="F159" t="s">
         <v>20</v>
@@ -4756,7 +4756,7 @@
         <v>159</v>
       </c>
       <c r="B160" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F160" t="s">
         <v>85</v>
@@ -4770,13 +4770,13 @@
         <v>160</v>
       </c>
       <c r="B161" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C161" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D161" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F161" t="s">
         <v>20</v>
@@ -4787,13 +4787,13 @@
         <v>161</v>
       </c>
       <c r="B162" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C162" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D162" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F162" t="s">
         <v>20</v>
@@ -4804,19 +4804,19 @@
         <v>162</v>
       </c>
       <c r="B163" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C163" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D163" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F163" t="s">
         <v>13</v>
       </c>
       <c r="J163" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.25">
@@ -4824,13 +4824,13 @@
         <v>163</v>
       </c>
       <c r="B164" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C164" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D164" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F164" t="s">
         <v>20</v>
@@ -4841,19 +4841,19 @@
         <v>164</v>
       </c>
       <c r="B165" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C165" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D165" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F165" t="s">
         <v>48</v>
       </c>
       <c r="J165" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.25">
@@ -4861,13 +4861,13 @@
         <v>165</v>
       </c>
       <c r="B166" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C166" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D166" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F166" t="s">
         <v>20</v>
@@ -4878,7 +4878,7 @@
         <v>166</v>
       </c>
       <c r="B167" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F167" t="s">
         <v>85</v>
@@ -4946,7 +4946,7 @@
         <v>56</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E1" s="10" t="s">
         <v>65</v>
@@ -4964,10 +4964,10 @@
         <v>80</v>
       </c>
       <c r="J1" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="K1" s="10" t="s">
         <v>207</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>208</v>
       </c>
       <c r="L1" s="10" t="s">
         <v>88</v>
@@ -4979,90 +4979,90 @@
         <v>97</v>
       </c>
       <c r="O1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="P1" s="1" t="s">
-        <v>128</v>
-      </c>
       <c r="Q1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="R1" s="1" t="s">
-        <v>144</v>
-      </c>
       <c r="S1" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="T1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B2" t="s">
         <v>161</v>
       </c>
-      <c r="B2" t="s">
-        <v>162</v>
-      </c>
       <c r="C2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D2">
         <v>3</v>
       </c>
       <c r="E2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F2" t="s">
         <v>210</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>211</v>
-      </c>
-      <c r="G2" t="s">
-        <v>212</v>
       </c>
       <c r="H2" t="s">
         <v>23</v>
       </c>
       <c r="I2" t="s">
+        <v>212</v>
+      </c>
+      <c r="J2" t="s">
         <v>213</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
+        <v>162</v>
+      </c>
+      <c r="L2" t="s">
+        <v>163</v>
+      </c>
+      <c r="M2" t="s">
         <v>214</v>
-      </c>
-      <c r="K2" t="s">
-        <v>163</v>
-      </c>
-      <c r="L2" t="s">
-        <v>164</v>
-      </c>
-      <c r="M2" t="s">
-        <v>215</v>
       </c>
       <c r="N2">
         <v>996289289004</v>
       </c>
       <c r="O2" t="s">
+        <v>345</v>
+      </c>
+      <c r="P2" t="s">
         <v>346</v>
       </c>
-      <c r="P2" t="s">
-        <v>347</v>
-      </c>
       <c r="Q2" t="s">
+        <v>345</v>
+      </c>
+      <c r="R2" t="s">
         <v>346</v>
       </c>
-      <c r="R2" t="s">
-        <v>347</v>
-      </c>
       <c r="S2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="T2" t="s">
+        <v>345</v>
+      </c>
+      <c r="U2" t="s">
         <v>346</v>
-      </c>
-      <c r="U2" t="s">
-        <v>347</v>
       </c>
     </row>
   </sheetData>
@@ -5081,71 +5081,71 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>167</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>169</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>171</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>173</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>175</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>177</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>178</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>179</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B9" s="3">
         <v>103</v>
@@ -5153,7 +5153,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B10" s="3">
         <v>15</v>
@@ -5161,7 +5161,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B11" s="3">
         <v>32</v>
@@ -5169,15 +5169,15 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>183</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>184</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B13" s="4">
         <v>46178</v>
@@ -5185,7 +5185,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B14" s="4">
         <v>46178</v>
@@ -5193,31 +5193,31 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>187</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>188</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>189</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>191</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B18" s="3">
         <v>4</v>
@@ -5225,18 +5225,18 @@
     </row>
     <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>194</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>195</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>196</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>197</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -5256,13 +5256,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>199</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -5270,10 +5270,10 @@
         <v>38</v>
       </c>
       <c r="B2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C2" t="s">
         <v>201</v>
-      </c>
-      <c r="C2" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -5281,10 +5281,10 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3" t="s">
         <v>203</v>
-      </c>
-      <c r="C3" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -5292,10 +5292,10 @@
         <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>